<commit_message>
feat: implement employee matching service with name-based fallback and update sample datasets
</commit_message>
<xml_diff>
--- a/samples/al-marwan-facilities-clean.xlsx
+++ b/samples/al-marwan-facilities-clean.xlsx
@@ -475,7 +475,7 @@
         <v>26</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -489,7 +489,7 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -517,7 +517,7 @@
         <v>26</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -531,7 +531,7 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -559,7 +559,7 @@
         <v>26</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -573,7 +573,7 @@
         <v>26</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement Gmail integration, add animation utilities, and update project dependencies and samples.
</commit_message>
<xml_diff>
--- a/samples/al-marwan-facilities-clean.xlsx
+++ b/samples/al-marwan-facilities-clean.xlsx
@@ -475,7 +475,7 @@
         <v>26</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -489,7 +489,7 @@
         <v>26</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -503,7 +503,7 @@
         <v>26</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -531,7 +531,7 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -545,7 +545,7 @@
         <v>26</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -573,7 +573,7 @@
         <v>26</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>